<commit_message>
feat: updated PCG graph. so now it goes from excel to csv to datatable back to PCG system in 1 pipeline
</commit_message>
<xml_diff>
--- a/Tools/manifest_tool/tests/module_list_BROKEN.xlsx
+++ b/Tools/manifest_tool/tests/module_list_BROKEN.xlsx
@@ -719,7 +719,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Residential_Block_Low</t>
+          <t>/Game/Meshes/Placeholders/SM_Cube.SM_Cube</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
@@ -773,7 +773,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Residential_Block_Mid</t>
+          <t>/Game/Meshes/Modules/SM_Residential_Block_Mid.SM_Residential_Block_Mid</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
@@ -831,7 +831,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Residential_Terrace</t>
+          <t>/Game/Meshes/Modules/SM_Residential_Terrace.SM_Residential_Terrace</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
@@ -889,7 +889,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Industrial_Warehouse</t>
+          <t>/Game/Meshes/Placeholders/SM_Cube.SM_Cube</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
@@ -947,7 +947,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Industrial_Processing</t>
+          <t>/Game/Meshes/Modules/SM_Industrial_Processing.SM_Industrial_Processing</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Service_Shopfront</t>
+          <t>/Game/Meshes/Placeholders/SM_Cube.SM_Cube</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Service_Utility_Block</t>
+          <t>/Game/Meshes/Modules/SM_Service_Utility_Block.SM_Service_Utility_Block</t>
         </is>
       </c>
       <c r="G8" s="3" t="n">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Hull_Rib_Straight</t>
+          <t>/Game/Meshes/Modules/SM_Hull_Rib_Straight.SM_Hull_Rib_Straight</t>
         </is>
       </c>
       <c r="G9" s="6" t="n">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Hull_Rib_Junction</t>
+          <t>/Game/Meshes/Modules/SM_Hull_Rib_Junction.SM_Hull_Rib_Junction</t>
         </is>
       </c>
       <c r="G10" s="6" t="n">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_DeckPlate_Standard</t>
+          <t>/Game/Meshes/Modules/SM_DeckPlate_Standard.SM_DeckPlate_Standard</t>
         </is>
       </c>
       <c r="G11" s="6" t="n">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_DeckPlate_Corner</t>
+          <t>/Game/Meshes/Modules/SM_DeckPlate_Corner.SM_DeckPlate_Corner</t>
         </is>
       </c>
       <c r="G12" s="6" t="n">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Truss_LoadBearing</t>
+          <t>/Game/Meshes/Modules/SM_Truss_LoadBearing.SM_Truss_LoadBearing</t>
         </is>
       </c>
       <c r="G13" s="6" t="n">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Bulkhead_Segment</t>
+          <t>/Game/Meshes/Modules/SM_Bulkhead_Segment.SM_Bulkhead_Segment</t>
         </is>
       </c>
       <c r="G14" s="6" t="n">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Ground_Paved_Street</t>
+          <t>/Game/Meshes/Modules/SM_Ground_Paved_Street.SM_Ground_Paved_Street</t>
         </is>
       </c>
       <c r="G15" s="9" t="n">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Ground_Paved_Plaza</t>
+          <t>/Game/Meshes/Modules/SM_Ground_Paved_Plaza.SM_Ground_Paved_Plaza</t>
         </is>
       </c>
       <c r="G16" s="9" t="n">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Ground_Planted_Grass</t>
+          <t>/Game/Meshes/Modules/SM_Ground_Planted_Grass.SM_Ground_Planted_Grass</t>
         </is>
       </c>
       <c r="G17" s="9" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Ground_Transition</t>
+          <t>/Game/Meshes/Modules/SM_Ground_Transition.SM_Ground_Transition</t>
         </is>
       </c>
       <c r="G18" s="9" t="n">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Pathway_Straight</t>
+          <t>/Game/Meshes/Modules/SM_Pathway_Straight.SM_Pathway_Straight</t>
         </is>
       </c>
       <c r="G19" s="9" t="n">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Tree_Deciduous_Large</t>
+          <t>/Game/Meshes/Modules/SM_Tree_Deciduous_Large.SM_Tree_Deciduous_Large</t>
         </is>
       </c>
       <c r="G20" s="12" t="n">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Tree_Deciduous_Small</t>
+          <t>/Game/Meshes/Placeholders/SM_Cube.SM_Cube</t>
         </is>
       </c>
       <c r="G21" s="12" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Tree_Conifer</t>
+          <t>/Game/Meshes/Modules/SM_Tree_Conifer.SM_Tree_Conifer</t>
         </is>
       </c>
       <c r="G22" s="12" t="n">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Shrub_Cluster</t>
+          <t>/Game/Meshes/Modules/SM_Shrub_Cluster.SM_Shrub_Cluster</t>
         </is>
       </c>
       <c r="G23" s="12" t="n">
@@ -1993,7 +1993,7 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_GroundCover_Grass</t>
+          <t>/Game/Meshes/Modules/SM_GroundCover_Grass.SM_GroundCover_Grass</t>
         </is>
       </c>
       <c r="G24" s="12" t="n">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_GroundCover_Fern</t>
+          <t>/Game/Meshes/Modules/SM_GroundCover_Fern.SM_GroundCover_Fern</t>
         </is>
       </c>
       <c r="G25" s="12" t="n">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Crop_Row_Agricultural</t>
+          <t>/Game/Meshes/Modules/SM_Crop_Row_Agricultural.SM_Crop_Row_Agricultural</t>
         </is>
       </c>
       <c r="G26" s="12" t="n">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="F28" s="14" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Pipe_Straight_Large</t>
+          <t>/Game/Meshes/Modules/SM_Pipe_Straight_Large.SM_Pipe_Straight_Large</t>
         </is>
       </c>
       <c r="G28" s="15" t="n">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="F30" s="14" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Vent_Wall_Mount</t>
+          <t>/Game/Meshes/Modules/SM_Vent_Wall_Mount.SM_Vent_Wall_Mount</t>
         </is>
       </c>
       <c r="G30" s="15" t="n">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_LightingRig_StreetLamp</t>
+          <t>/Game/Meshes/Modules/SM_Pipe_Elbow</t>
         </is>
       </c>
       <c r="G31" s="15" t="n">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="F32" s="14" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_LightingRig_OverheadStrip</t>
+          <t>/Game/Meshes/Modules/SM_LightingRig_OverheadStrip.SM_LightingRig_OverheadStrip</t>
         </is>
       </c>
       <c r="G32" s="15" t="n">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Cable_Conduit_Run</t>
+          <t>/Game/Meshes/Modules/SM_Vent_Wall_Mount.Wrong</t>
         </is>
       </c>
       <c r="G33" s="15" t="n">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_UtilityBox_Wall</t>
+          <t>/Game/Meshes/Modules/SM_UtilityBox_Wall.SM_UtilityBox_Wall</t>
         </is>
       </c>
       <c r="G34" s="15" t="n">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="F35" s="17" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Decal_RustStreak</t>
+          <t>/Game/Meshes/Modules/SM_Decal_RustStreak.SM_Decal_RustStreak</t>
         </is>
       </c>
       <c r="G35" s="18" t="n">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="F36" s="17" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Decal_Grime_Corner</t>
+          <t>/Game/Meshes/Modules/SM_Decal_Grime_Corner.SM_Decal_Grime_Corner</t>
         </is>
       </c>
       <c r="G36" s="18" t="n">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="F37" s="17" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Clutter_CrateStack</t>
+          <t>/Game/Meshes/Modules/SM_Clutter_CrateStack.SM_Clutter_CrateStack</t>
         </is>
       </c>
       <c r="G37" s="18" t="n">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="F38" s="17" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Mask_WeatheringOverlay</t>
+          <t>/Game/Meshes/Modules/SM_Mask_WeatheringOverlay.SM_Mask_WeatheringOverlay</t>
         </is>
       </c>
       <c r="G38" s="18" t="n">

</xml_diff>